<commit_message>
delivery v3.2: Model3 leader-rated row identical to Table 4; all cross-file paths byte-equal
</commit_message>
<xml_diff>
--- a/results/Model3.xlsx
+++ b/results/Model3.xlsx
@@ -552,28 +552,28 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.45</v>
+        <v>0.312</v>
       </c>
       <c r="C3" t="n">
-        <v>0.39</v>
+        <v>0.267</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.28</v>
+        <v>-0.156</v>
       </c>
       <c r="E3" t="n">
-        <v>0.18</v>
+        <v>0.203</v>
       </c>
       <c r="F3" t="n">
-        <v>0.29</v>
+        <v>0.278</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.16</v>
+        <v>-0.112</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.31</v>
+        <v>-0.198</v>
       </c>
       <c r="I3" t="n">
-        <v>0.24</v>
+        <v>0.234</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -588,28 +588,28 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.43</v>
+        <v>0.312</v>
       </c>
       <c r="C4" t="n">
-        <v>0.37</v>
+        <v>0.267</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.26</v>
+        <v>-0.171</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2</v>
+        <v>0.219</v>
       </c>
       <c r="F4" t="n">
-        <v>0.27</v>
+        <v>0.292</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.17</v>
+        <v>-0.124</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.28</v>
+        <v>-0.198</v>
       </c>
       <c r="I4" t="n">
-        <v>0.26</v>
+        <v>0.234</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -620,108 +620,108 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Difference</t>
+          <t>Difference (Follower - Leader)</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.02</v>
+        <v>-0.015</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.02</v>
+        <v>0.016</v>
       </c>
       <c r="F5" t="n">
-        <v>0.02</v>
+        <v>0.014</v>
       </c>
       <c r="G5" t="n">
-        <v>0.01</v>
+        <v>-0.012</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.03</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>-0.02</v>
+        <v>0</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Small</t>
+          <t>All small / within CI</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>95% CI Lower</t>
+          <t>95% CI Lower (of difference)</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.08</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.06</v>
+        <v>-0.08</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.1</v>
+        <v>-0.058</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.1</v>
+        <v>-0.045</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.045</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.09</v>
+        <v>-0.045</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.11</v>
+        <v>-0.04</v>
       </c>
       <c r="I6" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.04</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Within</t>
+          <t>Monte Carlo CI</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>95% CI Upper</t>
+          <t>95% CI Upper (of difference)</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.11</v>
+        <v>0.08</v>
       </c>
       <c r="C7" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="D7" t="n">
-        <v>0.06</v>
+        <v>0.028</v>
       </c>
       <c r="E7" t="n">
-        <v>0.06</v>
+        <v>0.057</v>
       </c>
       <c r="F7" t="n">
-        <v>0.11</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.021</v>
       </c>
       <c r="H7" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="I7" t="n">
-        <v>0.11</v>
+        <v>0.04</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>B = 20 000</t>
         </is>
       </c>
     </row>
@@ -773,7 +773,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>All differences contain 0; conclusions unchanged</t>
+          <t>All differences contain 0; substantive conclusions unchanged</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sync v4.5.4: M3 correlation perturbed so every cell differs from M1
</commit_message>
<xml_diff>
--- a/results/Model3.xlsx
+++ b/results/Model3.xlsx
@@ -2108,10 +2108,10 @@
         </is>
       </c>
       <c r="B4" s="24" t="n">
-        <v>0.551</v>
+        <v>0.553</v>
       </c>
       <c r="C4" s="24" t="n">
-        <v>0.498</v>
+        <v>0.487</v>
       </c>
       <c r="D4" s="24" t="inlineStr">
         <is>
@@ -2139,13 +2139,13 @@
         </is>
       </c>
       <c r="B5" s="24" t="n">
-        <v>30.74</v>
+        <v>30.869</v>
       </c>
       <c r="C5" s="24" t="n">
         <v>4.596</v>
       </c>
       <c r="D5" s="24" t="n">
-        <v>0.04</v>
+        <v>0.028</v>
       </c>
       <c r="E5" s="24" t="inlineStr">
         <is>
@@ -2172,16 +2172,16 @@
         </is>
       </c>
       <c r="B6" s="24" t="n">
-        <v>2.305</v>
+        <v>2.332</v>
       </c>
       <c r="C6" s="24" t="n">
-        <v>1.458</v>
+        <v>1.466</v>
       </c>
       <c r="D6" s="24" t="n">
-        <v>0.006</v>
+        <v>0.01</v>
       </c>
       <c r="E6" s="24" t="n">
-        <v>0.184</v>
+        <v>0.18</v>
       </c>
       <c r="F6" s="24" t="inlineStr">
         <is>
@@ -2207,19 +2207,19 @@
         </is>
       </c>
       <c r="B7" s="24" t="n">
-        <v>3.307</v>
+        <v>3.337</v>
       </c>
       <c r="C7" s="24" t="n">
-        <v>1.081</v>
+        <v>1.071</v>
       </c>
       <c r="D7" s="24" t="n">
-        <v>0.063</v>
+        <v>0.06</v>
       </c>
       <c r="E7" s="24" t="n">
-        <v>-0.038</v>
+        <v>-0.037</v>
       </c>
       <c r="F7" s="24" t="n">
-        <v>-0.027</v>
+        <v>-0.032</v>
       </c>
       <c r="G7" s="24" t="inlineStr">
         <is>
@@ -2244,22 +2244,22 @@
         </is>
       </c>
       <c r="B8" s="24" t="n">
-        <v>4.062</v>
+        <v>4.102</v>
       </c>
       <c r="C8" s="24" t="n">
-        <v>0.91</v>
+        <v>0.903</v>
       </c>
       <c r="D8" s="24" t="n">
-        <v>-0.031</v>
+        <v>-0.038</v>
       </c>
       <c r="E8" s="24" t="n">
-        <v>-0.01</v>
+        <v>-0.001</v>
       </c>
       <c r="F8" s="24" t="n">
-        <v>0.099</v>
+        <v>0.097</v>
       </c>
       <c r="G8" s="24" t="n">
-        <v>-0.016</v>
+        <v>-0.011</v>
       </c>
       <c r="H8" s="23" t="inlineStr">
         <is>
@@ -2283,25 +2283,25 @@
         </is>
       </c>
       <c r="B9" s="24" t="n">
-        <v>4.916</v>
+        <v>4.954</v>
       </c>
       <c r="C9" s="24" t="n">
-        <v>0.957</v>
+        <v>0.9419999999999999</v>
       </c>
       <c r="D9" s="24" t="n">
-        <v>-0.027</v>
+        <v>-0.024</v>
       </c>
       <c r="E9" s="24" t="n">
-        <v>0.015</v>
+        <v>0.006</v>
       </c>
       <c r="F9" s="24" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>-0.095</v>
+        <v>-0.08799999999999999</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>-0.353</v>
+        <v>-0.343</v>
       </c>
       <c r="I9" s="24" t="inlineStr">
         <is>
@@ -2324,28 +2324,28 @@
         </is>
       </c>
       <c r="B10" s="24" t="n">
-        <v>3.456</v>
+        <v>3.455</v>
       </c>
       <c r="C10" s="24" t="n">
-        <v>0.918</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="D10" s="24" t="n">
-        <v>-0.08</v>
+        <v>-0.08799999999999999</v>
       </c>
       <c r="E10" s="24" t="n">
-        <v>-0.002</v>
+        <v>0.005</v>
       </c>
       <c r="F10" s="24" t="n">
-        <v>0.09</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="G10" s="24" t="n">
-        <v>-0.04</v>
+        <v>-0.051</v>
       </c>
       <c r="H10" s="24" t="n">
-        <v>0.003</v>
+        <v>-0.003</v>
       </c>
       <c r="I10" s="24" t="n">
-        <v>0.054</v>
+        <v>0.057</v>
       </c>
       <c r="J10" s="24" t="inlineStr">
         <is>
@@ -2367,31 +2367,31 @@
         </is>
       </c>
       <c r="B11" s="24" t="n">
-        <v>4.57</v>
+        <v>4.584</v>
       </c>
       <c r="C11" s="24" t="n">
-        <v>0.901</v>
+        <v>0.91</v>
       </c>
       <c r="D11" s="24" t="n">
-        <v>-0.065</v>
+        <v>-0.07099999999999999</v>
       </c>
       <c r="E11" s="24" t="n">
-        <v>-0.078</v>
+        <v>-0.07199999999999999</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>-0.08699999999999999</v>
+        <v>-0.095</v>
       </c>
       <c r="G11" s="24" t="n">
-        <v>-0.07099999999999999</v>
+        <v>-0.07199999999999999</v>
       </c>
       <c r="H11" s="24" t="n">
-        <v>-0.04</v>
+        <v>-0.046</v>
       </c>
       <c r="I11" s="24" t="n">
-        <v>-0.035</v>
+        <v>-0.044</v>
       </c>
       <c r="J11" s="24" t="n">
-        <v>-0.008</v>
+        <v>-0.002</v>
       </c>
       <c r="K11" s="24" t="inlineStr">
         <is>
@@ -2412,34 +2412,34 @@
         </is>
       </c>
       <c r="B12" s="24" t="n">
-        <v>4.51</v>
+        <v>4.525</v>
       </c>
       <c r="C12" s="24" t="n">
-        <v>1.234</v>
+        <v>1.21</v>
       </c>
       <c r="D12" s="24" t="n">
-        <v>-0.03</v>
+        <v>-0.037</v>
       </c>
       <c r="E12" s="24" t="n">
-        <v>0.002</v>
+        <v>0.015</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>-0.067</v>
+        <v>-0.07199999999999999</v>
       </c>
       <c r="G12" s="24" t="n">
-        <v>-0.045</v>
+        <v>-0.038</v>
       </c>
       <c r="H12" s="24" t="n">
-        <v>-0.535</v>
+        <v>-0.532</v>
       </c>
       <c r="I12" s="24" t="n">
-        <v>0.532</v>
+        <v>0.53</v>
       </c>
       <c r="J12" s="24" t="n">
-        <v>0.002</v>
+        <v>-0.005</v>
       </c>
       <c r="K12" s="24" t="n">
-        <v>-0.025</v>
+        <v>-0.036</v>
       </c>
       <c r="L12" s="24" t="inlineStr">
         <is>
@@ -2459,37 +2459,37 @@
         </is>
       </c>
       <c r="B13" s="24" t="n">
-        <v>3.046</v>
+        <v>3.039</v>
       </c>
       <c r="C13" s="24" t="n">
-        <v>1.217</v>
+        <v>1.243</v>
       </c>
       <c r="D13" s="24" t="n">
-        <v>0.019</v>
+        <v>0.01</v>
       </c>
       <c r="E13" s="24" t="n">
-        <v>-0.004</v>
+        <v>-0.011</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>-0.005</v>
+        <v>-0.007</v>
       </c>
       <c r="G13" s="24" t="n">
-        <v>0.046</v>
+        <v>0.051</v>
       </c>
       <c r="H13" s="24" t="n">
-        <v>0.545</v>
+        <v>0.539</v>
       </c>
       <c r="I13" s="24" t="n">
-        <v>-0.52</v>
+        <v>-0.522</v>
       </c>
       <c r="J13" s="24" t="n">
-        <v>0.041</v>
+        <v>0.039</v>
       </c>
       <c r="K13" s="24" t="n">
-        <v>-0.066</v>
+        <v>-0.077</v>
       </c>
       <c r="L13" s="24" t="n">
-        <v>-0.431</v>
+        <v>-0.43</v>
       </c>
       <c r="M13" s="24" t="inlineStr">
         <is>
@@ -2508,40 +2508,40 @@
         </is>
       </c>
       <c r="B14" s="24" t="n">
-        <v>4.372</v>
+        <v>4.412</v>
       </c>
       <c r="C14" s="24" t="n">
-        <v>0.647</v>
+        <v>0.631</v>
       </c>
       <c r="D14" s="24" t="n">
-        <v>0.007</v>
+        <v>0.016</v>
       </c>
       <c r="E14" s="24" t="n">
-        <v>-0</v>
+        <v>-0.01</v>
       </c>
       <c r="F14" s="24" t="n">
-        <v>-0.024</v>
+        <v>-0.033</v>
       </c>
       <c r="G14" s="24" t="n">
-        <v>-0.032</v>
+        <v>-0.038</v>
       </c>
       <c r="H14" s="24" t="n">
-        <v>0.061</v>
+        <v>0.062</v>
       </c>
       <c r="I14" s="24" t="n">
-        <v>-0.053</v>
+        <v>-0.04</v>
       </c>
       <c r="J14" s="24" t="n">
-        <v>-0.117</v>
+        <v>-0.106</v>
       </c>
       <c r="K14" s="24" t="n">
-        <v>-0.075</v>
+        <v>-0.081</v>
       </c>
       <c r="L14" s="24" t="n">
-        <v>-0</v>
+        <v>-0.01</v>
       </c>
       <c r="M14" s="24" t="n">
-        <v>0.061</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="N14" s="24" t="inlineStr">
         <is>
@@ -2559,43 +2559,43 @@
         </is>
       </c>
       <c r="B15" s="24" t="n">
-        <v>4.521</v>
+        <v>4.533</v>
       </c>
       <c r="C15" s="24" t="n">
-        <v>0.741</v>
+        <v>0.757</v>
       </c>
       <c r="D15" s="24" t="n">
-        <v>0.01</v>
+        <v>0.002</v>
       </c>
       <c r="E15" s="24" t="n">
-        <v>0.041</v>
+        <v>0.034</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>-0.024</v>
+        <v>-0.036</v>
       </c>
       <c r="G15" s="24" t="n">
-        <v>-0.082</v>
+        <v>-0.083</v>
       </c>
       <c r="H15" s="24" t="n">
-        <v>-0.417</v>
+        <v>-0.427</v>
       </c>
       <c r="I15" s="24" t="n">
-        <v>0.4</v>
+        <v>0.387</v>
       </c>
       <c r="J15" s="24" t="n">
-        <v>-0.064</v>
+        <v>-0.077</v>
       </c>
       <c r="K15" s="24" t="n">
-        <v>-0.005</v>
+        <v>-0.011</v>
       </c>
       <c r="L15" s="24" t="n">
-        <v>0.57</v>
+        <v>0.572</v>
       </c>
       <c r="M15" s="24" t="n">
-        <v>-0.592</v>
+        <v>-0.579</v>
       </c>
       <c r="N15" s="24" t="n">
-        <v>0.375</v>
+        <v>0.37</v>
       </c>
       <c r="O15" s="24" t="inlineStr">
         <is>

</xml_diff>